<commit_message>
galeras updated con nuevos iso
</commit_message>
<xml_diff>
--- a/Galeras/Galeras_cellulose.xlsx
+++ b/Galeras/Galeras_cellulose.xlsx
@@ -3118,7 +3118,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>jh-3621</t>
+          <t>jh-p50-3621</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>jh-3657</t>
+          <t>jh-p60-3657</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -3238,7 +3238,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>jh-2070</t>
+          <t>jh-p24-2070</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>jh-2053</t>
+          <t>jh-p22-2053</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>jh-3600</t>
+          <t>jh-p28-3600</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>jh-2034</t>
+          <t>jh-p23-2034</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -3468,7 +3468,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>jh-3620</t>
+          <t>jh-p50-3620</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -3531,7 +3531,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>jh-3710</t>
+          <t>jh-p48-3710</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -3594,7 +3594,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>jh-2531</t>
+          <t>jh-p62-2531</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>jh-2525</t>
+          <t>jh-p60-2525</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>jh-2456</t>
+          <t>jh-p48-2456</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -3777,7 +3777,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>jh-3625</t>
+          <t>jh-p50-3625</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>jh-3698</t>
+          <t>jh-p48-3698</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -3903,7 +3903,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>jh-3623</t>
+          <t>jh-p50-3623</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>jh-3659</t>
+          <t>jh-p60-3659</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>jh-2529</t>
+          <t>jh-p62-2529</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>jh-3608</t>
+          <t>jh-p62-3608</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -4149,7 +4149,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>jh-3582</t>
+          <t>jh-p28-3582</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>jh-3706</t>
+          <t>jh-p48-3706</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>jh-3607</t>
+          <t>jh-p62-3607</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -4338,7 +4338,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>jh-3580</t>
+          <t>jh-p28-3580</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>jh-3696</t>
+          <t>jh-p48-3696</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -4460,7 +4460,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>jh-3703</t>
+          <t>jh-p48-3703</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>jh-3662</t>
+          <t>jh-p60-3662</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -4578,7 +4578,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>jh-3601</t>
+          <t>jh-p28-3601</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -4637,7 +4637,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>jh-3579</t>
+          <t>jh-p28-3579</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>jh-3589</t>
+          <t>jh-p28-3589</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -4763,7 +4763,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>jh-3707</t>
+          <t>jh-p48-3707</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4826,7 +4826,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>jh-3611</t>
+          <t>jh-p62-3611</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>jh-3595</t>
+          <t>jh-p62-3595</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -4936,7 +4936,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>jh-3581</t>
+          <t>jh-p28-3581</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -4999,7 +4999,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>jh-3609</t>
+          <t>jh-p62-3609</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>jh-3659</t>
+          <t>jh-p60-3659</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -5117,7 +5117,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>jh-3697</t>
+          <t>jh-p48-3697</t>
         </is>
       </c>
       <c r="C77" t="n">

</xml_diff>